<commit_message>
Se agrega el avance de la campaña dinámica
</commit_message>
<xml_diff>
--- a/00_Administración/presupuesto_banco_ensayos.xlsx
+++ b/00_Administración/presupuesto_banco_ensayos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josei\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udeconce-my.sharepoint.com/personal/joarriagada2021_udec_cl/Documents/Escritorio/Memoria/00_Administración/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A087F001-3914-46A3-8F91-971FE9E8414F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{A087F001-3914-46A3-8F91-971FE9E8414F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7785E24-2004-4893-9BB7-FDCCF43C2850}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -193,7 +193,7 @@
     <numFmt numFmtId="164" formatCode="\$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0\x"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -266,6 +266,14 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -317,10 +325,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -359,8 +368,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -927,7 +940,7 @@
         <f>B18*C18</f>
         <v>9082</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="20" t="s">
         <v>33</v>
       </c>
       <c r="F18" s="8" t="s">

</xml_diff>